<commit_message>
default headers to bold (#121)
</commit_message>
<xml_diff>
--- a/src/ExcelsiorAspose.Tests/ColumnAttributeTests.Test.verified.xlsx
+++ b/src/ExcelsiorAspose.Tests/ColumnAttributeTests.Test.verified.xlsx
@@ -54,8 +54,15 @@
     <numFmt numFmtId="177" formatCode="yyyy-MM-dd"/>
     <numFmt numFmtId="178" formatCode="0000"/>
   </numFmts>
-  <fonts count="1">
+  <fonts count="2">
     <font>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
       <sz val="10"/>
       <color theme="1"/>
       <name val="Arial"/>
@@ -90,8 +97,9 @@
     <xf numFmtId="43" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="41" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="178" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
@@ -489,51 +497,51 @@
   <dimension ref="A1:D3"/>
   <sheetFormatPr defaultRowHeight="12.75"/>
   <cols>
-    <col min="1" max="1" width="15.7142857142857" customWidth="1"/>
+    <col min="1" max="1" width="16.7142857142857" customWidth="1"/>
     <col min="2" max="2" width="20.7142857142857" customWidth="1"/>
-    <col min="3" max="3" width="12.7142857142857" customWidth="1"/>
+    <col min="3" max="3" width="13.7142857142857" customWidth="1"/>
     <col min="4" max="4" width="30.7142857142857" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="14" customHeight="1">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="2" spans="1:4" ht="14" customHeight="1">
-      <c r="A2" s="1">
+      <c r="A2" s="2">
         <v>1</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="B2" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="C2" s="3">
+      <c r="C2" s="4">
         <v>43845</v>
       </c>
-      <c r="D2" s="2" t="s">
+      <c r="D2" s="3" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="3" spans="1:4" ht="14" customHeight="1">
-      <c r="A3" s="1">
+      <c r="A3" s="2">
         <v>2</v>
       </c>
-      <c r="B3" s="2" t="s">
+      <c r="B3" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="C3" s="2" t="s">
+      <c r="C3" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="D3" s="2" t="s">
+      <c r="D3" s="3" t="s">
         <v>8</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Round row to nearest 5 since Aspose AutoFitRows is not deterministic
</commit_message>
<xml_diff>
--- a/src/ExcelsiorAspose.Tests/ColumnAttributeTests.Test.verified.xlsx
+++ b/src/ExcelsiorAspose.Tests/ColumnAttributeTests.Test.verified.xlsx
@@ -503,7 +503,7 @@
     <col min="4" max="4" width="30.7142857142857" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="14" customHeight="1">
+    <row r="1" spans="1:4" ht="16" customHeight="1">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -517,7 +517,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:4" ht="14" customHeight="1">
+    <row r="2" spans="1:4" ht="16" customHeight="1">
       <c r="A2" s="2">
         <v>1</v>
       </c>
@@ -531,7 +531,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="3" spans="1:4" ht="14" customHeight="1">
+    <row r="3" spans="1:4" ht="16" customHeight="1">
       <c r="A3" s="2">
         <v>2</v>
       </c>

</xml_diff>